<commit_message>
Fix I-22: 4 mm inserts in the back cover leave a 2.5 mm floor
The four NEMA17-mount M3 insert holes were 6 deep from the motor face
of the 14 mm back cover, leaving 1.0 mm over the Ø72 x 7 carrier
recess. They are now 4.5 deep for the short ruthex M3S x 4.0 (same
knurl as the M3 x 5.7, so FIT.insert_m3 is unchanged), leaving 2.5 mm.

The short insert is not stocked: inventory.md and inventory.xlsx list
it to order, and the mount screws must be M3 x 14 (M3 x 16 bottoms
out). The back cover is recorded as a gate departure.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$5:$N$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$5:$N$78</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Inventory'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N80"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -612,6 +612,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -1822,14 +1823,14 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>FIT.insert_m3: ring gear (12), back cover (4), carrier plates (6), Wall (9 per segment), Base/Top proximal (4 per segment)</t>
+          <t>FIT.insert_m3: ring gear (12), carrier plates (6), Wall (9 per segment), Base/Top proximal (4 per segment). Back cover: M3 × 4, next row (I-22)</t>
         </is>
       </c>
       <c r="H28" s="6" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>432</v>
+        <v>396</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -1844,7 +1845,7 @@
       </c>
       <c r="N28" s="6" t="inlineStr">
         <is>
-          <t>Approximate (~48 per arm)</t>
+          <t>Approximate (~44 per arm)</t>
         </is>
       </c>
     </row>
@@ -1854,37 +1855,35 @@
           <t>Arm: fasteners and threaded inserts (consumables)</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>ruthex M5 × 9.5 heat-set insert (50-pack)</t>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>ruthex M3S × 4.0 short heat-set insert (100-pack) — TO ORDER</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>B07YSVXWS8</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>Not bought yet</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>9.99</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F29" s="8" t="n"/>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>FIT.insert_m5: box bottom (7)</t>
+          <t>FIT.insert_m3: back cover, NEMA17 mount (4); 4.5 mm holes leave 2.5 mm over the carrier recess (design.md I-22)</t>
         </is>
       </c>
       <c r="H29" s="6" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -1897,7 +1896,11 @@
         <f>IF(K29="","",MAX(0,I29-K29))</f>
         <v/>
       </c>
-      <c r="N29" s="6" t="inlineStr"/>
+      <c r="N29" s="6" t="inlineStr">
+        <is>
+          <t>Not on Amazon: 3DJake US, ruthex GE-M3Sx40-002 (EAN 4260528721238). Same knurl as M3 × 5.7 (Ø4.6, Ø4.0 hole). Screws: M3 × 14 (not 16)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1907,41 +1910,46 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>FFVRVSS brass insert assortment M2–M5 (328 pc) with heat-set tool</t>
+          <t>ruthex M5 × 9.5 heat-set insert (50-pack)</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>B0FH4JQ3VB</t>
+          <t>B07YSVXWS8</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n"/>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>50</v>
+      </c>
       <c r="F30" s="8" t="n">
-        <v>6.92</v>
+        <v>9.99</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>Insert tips for soldering irons; spare inserts</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
+          <t>FIT.insert_m5: box bottom (7)</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>63</v>
+      </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>kits</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="10" t="n"/>
-      <c r="M30" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M30" s="11">
+        <f>IF(K30="","",MAX(0,I30-K30))</f>
+        <v/>
       </c>
       <c r="N30" s="6" t="inlineStr"/>
     </row>
@@ -1953,52 +1961,43 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>iexcell M3 × 8 button head, 12.9 (100-pack)</t>
+          <t>FFVRVSS brass insert assortment M2–M5 (328 pc) with heat-set tool</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>B0CP4B16KF</t>
+          <t>B0FH4JQ3VB</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>2 packs = 200</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>200</v>
-      </c>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n"/>
       <c r="F31" s="8" t="n">
-        <v>17.72</v>
+        <v>6.92</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>M3 screws (lengths not recorded)</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="n">
-        <v>75</v>
-      </c>
-      <c r="I31" s="6" t="n">
-        <v>675</v>
-      </c>
+          <t>Insert tips for soldering irons; spare inserts</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>kits</t>
         </is>
       </c>
       <c r="K31" s="9" t="n"/>
       <c r="L31" s="10" t="n"/>
-      <c r="M31" s="11">
-        <f>IF(COUNT(K31,K32,K33,K34)=0,"",MAX(0,I31-SUM(K31,K32,K33,K34)))</f>
-        <v/>
-      </c>
-      <c r="N31" s="6" t="inlineStr">
-        <is>
-          <t>Need covers all M3 button heads (8, 10, 12, 16 mm) together; to-order compares it with the four rows' counts</t>
-        </is>
-      </c>
+      <c r="M31" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -2008,39 +2007,35 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>iexcell M3 × 10 button head, 12.9 (100-pack)</t>
+          <t>iexcell M3 × 8 button head, 12.9 (100-pack)</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>B0CP4BLD7Z</t>
+          <t>B0CP4B16KF</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2 packs = 200</t>
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>8.859999999999999</v>
+        <v>17.72</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
           <t>M3 screws (lengths not recorded)</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>(shared, see first row)</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>(shared, see first row)</t>
-        </is>
+      <c r="H32" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>675</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -2049,12 +2044,15 @@
       </c>
       <c r="K32" s="9" t="n"/>
       <c r="L32" s="10" t="n"/>
-      <c r="M32" s="14" t="inlineStr">
-        <is>
-          <t>see first row</t>
-        </is>
-      </c>
-      <c r="N32" s="6" t="inlineStr"/>
+      <c r="M32" s="11">
+        <f>IF(COUNT(K32,K33,K34,K35)=0,"",MAX(0,I32-SUM(K32,K33,K34,K35)))</f>
+        <v/>
+      </c>
+      <c r="N32" s="6" t="inlineStr">
+        <is>
+          <t>Need covers all M3 button heads (8, 10, 12, 16 mm) together; to-order compares it with the four rows' counts</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2064,24 +2062,24 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>iexcell M3 × 12 button head, 12.9 (100-pack)</t>
+          <t>iexcell M3 × 10 button head, 12.9 (100-pack)</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>B0CP4B65CC</t>
+          <t>B0CP4BLD7Z</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>2 packs = 200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>17.72</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -2120,12 +2118,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>iexcell M3 × 16 button head, 12.9 (100-pack)</t>
+          <t>iexcell M3 × 12 button head, 12.9 (100-pack)</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>B0CP48RN8K</t>
+          <t>B0CP4B65CC</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2137,7 +2135,7 @@
         <v>200</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>17.92</v>
+        <v>17.72</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
@@ -2176,50 +2174,53 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Kadrick M3 assortment, 4–35 mm, with nuts and washers (2240 pc)</t>
+          <t>iexcell M3 × 16 button head, 12.9 (100-pack)</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>B0CQNN6NY3</t>
+          <t>B0CP48RN8K</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="n"/>
+          <t>2 packs = 200</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>200</v>
+      </c>
       <c r="F35" s="8" t="n">
-        <v>22.99</v>
+        <v>17.92</v>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Includes M3 × 35 for the idler jack screws (purchased/socket_head_m3x35.py, 2 per segment)</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I35" s="6" t="n">
-        <v>36</v>
+          <t>M3 screws (lengths not recorded)</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>(shared, see first row)</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>(shared, see first row)</t>
+        </is>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>M3 × 35 screws</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K35" s="9" t="n"/>
       <c r="L35" s="10" t="n"/>
-      <c r="M35" s="11">
-        <f>IF(K35="","",MAX(0,I35-K35))</f>
-        <v/>
-      </c>
-      <c r="N35" s="6" t="inlineStr">
-        <is>
-          <t>Count the M3 × 35 socket heads left in the kit</t>
-        </is>
-      </c>
+      <c r="M35" s="14" t="inlineStr">
+        <is>
+          <t>see first row</t>
+        </is>
+      </c>
+      <c r="N35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -2229,28 +2230,26 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>M5 × 40 button head, black oxide SS (25-pack)</t>
+          <t>Kadrick M3 assortment, 4–35 mm, with nuts and washers (2240 pc)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>B0GJJBQDCD</t>
+          <t>B0CQNN6NY3</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>2 packs = 50</t>
-        </is>
-      </c>
-      <c r="E36" s="6" t="n">
-        <v>50</v>
-      </c>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n"/>
       <c r="F36" s="8" t="n">
-        <v>17.36</v>
+        <v>22.99</v>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>purchased/button_head_m5x40.py: idler axles (2 per segment)</t>
+          <t>Includes M3 × 35 for the idler jack screws (purchased/socket_head_m3x35.py, 2 per segment)</t>
         </is>
       </c>
       <c r="H36" s="6" t="n">
@@ -2261,7 +2260,7 @@
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>M3 × 35 screws</t>
         </is>
       </c>
       <c r="K36" s="9" t="n"/>
@@ -2270,7 +2269,11 @@
         <f>IF(K36="","",MAX(0,I36-K36))</f>
         <v/>
       </c>
-      <c r="N36" s="6" t="inlineStr"/>
+      <c r="N36" s="6" t="inlineStr">
+        <is>
+          <t>Count the M3 × 35 socket heads left in the kit</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -2280,28 +2283,28 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>M5 × 45 button head (25-pack)</t>
+          <t>M5 × 40 button head, black oxide SS (25-pack)</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>B0GJJKXJG5</t>
+          <t>B0GJJBQDCD</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>2 packs = 50</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>8.68</v>
+        <v>17.36</v>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Probably the J1 pulley–hinge clamp (4 × M5, length not recorded)</t>
+          <t>purchased/button_head_m5x40.py: idler axles (2 per segment)</t>
         </is>
       </c>
       <c r="H37" s="6" t="n">
@@ -2318,14 +2321,10 @@
       <c r="K37" s="9" t="n"/>
       <c r="L37" s="10" t="n"/>
       <c r="M37" s="11">
-        <f>IF(COUNT(K37,K38)=0,"",MAX(0,I37-SUM(K37,K38)))</f>
+        <f>IF(K37="","",MAX(0,I37-K37))</f>
         <v/>
       </c>
-      <c r="N37" s="6" t="inlineStr">
-        <is>
-          <t>J1 pulley–hinge clamp length not recorded: need covers M5 × 45 and M5 × 50 together</t>
-        </is>
-      </c>
+      <c r="N37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -2335,12 +2334,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>M5 × 50 button head (25-pack)</t>
+          <t>M5 × 45 button head (25-pack)</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>B0GJJDKQLZ</t>
+          <t>B0GJJKXJG5</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2359,15 +2358,11 @@
           <t>Probably the J1 pulley–hinge clamp (4 × M5, length not recorded)</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>(shared, see first row)</t>
-        </is>
-      </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>(shared, see first row)</t>
-        </is>
+      <c r="H38" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>36</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -2376,12 +2371,15 @@
       </c>
       <c r="K38" s="9" t="n"/>
       <c r="L38" s="10" t="n"/>
-      <c r="M38" s="14" t="inlineStr">
-        <is>
-          <t>see first row</t>
-        </is>
-      </c>
-      <c r="N38" s="6" t="inlineStr"/>
+      <c r="M38" s="11">
+        <f>IF(COUNT(K38,K39)=0,"",MAX(0,I38-SUM(K38,K39)))</f>
+        <v/>
+      </c>
+      <c r="N38" s="6" t="inlineStr">
+        <is>
+          <t>J1 pulley–hinge clamp length not recorded: need covers M5 × 45 and M5 × 50 together</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -2391,50 +2389,53 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Kadrick M5 assortment, 8–40 mm, with nuts and washers (960 pc)</t>
+          <t>M5 × 50 button head (25-pack)</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>B0DRCBVH8K</t>
+          <t>B0GJJDKQLZ</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="n"/>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>25</v>
+      </c>
       <c r="F39" s="8" t="n">
-        <v>22.99</v>
+        <v>8.68</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Box top–bottom screws (7), M5 nuts for the idler axles (purchased/hex_nut_m5.py, 2 per segment)</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="I39" s="6" t="n">
-        <v>63</v>
+          <t>Probably the J1 pulley–hinge clamp (4 × M5, length not recorded)</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>(shared, see first row)</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>(shared, see first row)</t>
+        </is>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>M5 screws</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K39" s="9" t="n"/>
       <c r="L39" s="10" t="n"/>
-      <c r="M39" s="11">
-        <f>IF(K39="","",MAX(0,I39-K39))</f>
-        <v/>
-      </c>
-      <c r="N39" s="6" t="inlineStr">
-        <is>
-          <t>Also supplies the idler-axle M5 nuts: 4 per arm, 36 for 9 sets (count those too)</t>
-        </is>
-      </c>
+      <c r="M39" s="14" t="inlineStr">
+        <is>
+          <t>see first row</t>
+        </is>
+      </c>
+      <c r="N39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -2444,39 +2445,37 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>ZDingTech M4 × 5 set screw (110-pack)</t>
+          <t>Kadrick M5 assortment, 8–40 mm, with nuts and washers (960 pc)</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>B0CF299SDT</t>
+          <t>B0DRCBVH8K</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>110</t>
-        </is>
-      </c>
-      <c r="E40" s="6" t="n">
-        <v>110</v>
-      </c>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n"/>
       <c r="F40" s="8" t="n">
-        <v>6.69</v>
+        <v>22.99</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Probably the gearbox input-shaft set screw (Ø4 cross hole)</t>
+          <t>Box top–bottom screws (7), M5 nuts for the idler axles (purchased/hex_nut_m5.py, 2 per segment)</t>
         </is>
       </c>
       <c r="H40" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>9</v>
+        <v>63</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>M5 screws</t>
         </is>
       </c>
       <c r="K40" s="9" t="n"/>
@@ -2485,7 +2484,11 @@
         <f>IF(K40="","",MAX(0,I40-K40))</f>
         <v/>
       </c>
-      <c r="N40" s="6" t="inlineStr"/>
+      <c r="N40" s="6" t="inlineStr">
+        <is>
+          <t>Also supplies the idler-axle M5 nuts: 4 per arm, 36 for 9 sets (count those too)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -2495,88 +2498,92 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>304 SS flat washer assortment M2–M12 (1100 pc)</t>
+          <t>ZDingTech M4 × 5 set screw (110-pack)</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>B0DZ5H9T4Z</t>
+          <t>B0CF299SDT</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E41" s="6" t="n"/>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>110</v>
+      </c>
       <c r="F41" s="8" t="n">
-        <v>6.99</v>
+        <v>6.69</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="n"/>
-      <c r="I41" s="6" t="n"/>
+          <t>Probably the gearbox input-shaft set screw (Ø4 cross hole)</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>kits</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K41" s="9" t="n"/>
       <c r="L41" s="10" t="n"/>
-      <c r="M41" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M41" s="11">
+        <f>IF(K41="","",MAX(0,I41-K41))</f>
+        <v/>
       </c>
       <c r="N41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Electronics</t>
+          <t>Arm: fasteners and threaded inserts (consumables)</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Arduino Uno Q</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>304 SS flat washer assortment M2–M12 (1100 pc)</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>B0DZ5H9T4Z</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Arduino store (not Amazon): fill in</t>
+          <t>1 kit</t>
         </is>
       </c>
       <c r="E42" s="6" t="n"/>
-      <c r="F42" s="8" t="n"/>
+      <c r="F42" s="8" t="n">
+        <v>6.99</v>
+      </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Controller</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="6" t="n">
-        <v>9</v>
-      </c>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
       <c r="J42" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>kits</t>
         </is>
       </c>
       <c r="K42" s="9" t="n"/>
       <c r="L42" s="10" t="n"/>
-      <c r="M42" s="11">
-        <f>IF(K42="","",MAX(0,I42-K42))</f>
-        <v/>
+      <c r="M42" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N42" s="6" t="inlineStr"/>
     </row>
@@ -2588,28 +2595,24 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>ACEIRMC CNC Shield V3 kit with 4 × A4988 and heat sinks</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>B07TT3C3HB</t>
+          <t>Arduino Uno Q</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>6 kits (6 shields, 24 A4988)</t>
-        </is>
-      </c>
-      <c r="E43" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F43" s="8" t="n">
-        <v>58.14</v>
-      </c>
+          <t>Arduino store (not Amazon): fill in</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="8" t="n"/>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Drives the 4 steppers (UNO header). Check that it fits the Uno Q</t>
+          <t>Controller</t>
         </is>
       </c>
       <c r="H43" s="6" t="n">
@@ -2620,7 +2623,7 @@
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
-          <t>shields</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K43" s="9" t="n"/>
@@ -2639,43 +2642,46 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>HiLetgo A4988 driver with heat sink (5-pack)</t>
+          <t>ACEIRMC CNC Shield V3 kit with 4 × A4988 and heat sinks</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>B07BND65C8</t>
+          <t>B07TT3C3HB</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>3 packs = 15</t>
+          <t>6 kits (6 shields, 24 A4988)</t>
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>29.04</v>
+        <v>58.14</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>Phase 1 breadboard wiring; spares for the shields</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="6" t="n"/>
+          <t>Drives the 4 steppers (UNO header). Check that it fits the Uno Q</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>shields</t>
         </is>
       </c>
       <c r="K44" s="9" t="n"/>
       <c r="L44" s="10" t="n"/>
-      <c r="M44" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M44" s="11">
+        <f>IF(K44="","",MAX(0,I44-K44))</f>
+        <v/>
       </c>
       <c r="N44" s="6" t="inlineStr"/>
     </row>
@@ -2687,36 +2693,32 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>MG996R metal-gear servo (6-pack)</t>
+          <t>HiLetgo A4988 driver with heat sink (5-pack)</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>B0BMM1G74B</t>
+          <t>B07BND65C8</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3 packs = 15</t>
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>26.98</v>
+        <v>29.04</v>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Handout SERVO_PIN; gripper/end effector</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I45" s="6" t="n">
-        <v>9</v>
-      </c>
+          <t>Phase 1 breadboard wiring; spares for the shields</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
       <c r="J45" s="6" t="inlineStr">
         <is>
           <t>units</t>
@@ -2724,9 +2726,10 @@
       </c>
       <c r="K45" s="9" t="n"/>
       <c r="L45" s="10" t="n"/>
-      <c r="M45" s="11">
-        <f>IF(K45="","",MAX(0,I45-K45))</f>
-        <v/>
+      <c r="M45" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N45" s="6" t="inlineStr"/>
     </row>
@@ -2738,32 +2741,36 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>SG90 9 g micro servo (5-pack)</t>
+          <t>MG996R metal-gear servo (6-pack)</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>B0BJQ2QTHG</t>
+          <t>B0BMM1G74B</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>9.98</v>
+        <v>26.98</v>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>Light-duty servo (handout §2 table)</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="6" t="n"/>
+          <t>Handout SERVO_PIN; gripper/end effector</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
           <t>units</t>
@@ -2771,10 +2778,9 @@
       </c>
       <c r="K46" s="9" t="n"/>
       <c r="L46" s="10" t="n"/>
-      <c r="M46" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M46" s="11">
+        <f>IF(K46="","",MAX(0,I46-K46))</f>
+        <v/>
       </c>
       <c r="N46" s="6" t="inlineStr"/>
     </row>
@@ -2786,36 +2792,32 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>URBEST roller-lever micro switch, SPDT (10-pack)</t>
+          <t>SG90 9 g micro servo (5-pack)</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>B00MFRMFS6</t>
+          <t>B0BJQ2QTHG</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>4 packs = 40</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E47" s="6" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>27.96</v>
+        <v>9.98</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Handout LIMIT_SWITCH_PIN; joint homing</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I47" s="6" t="n">
-        <v>36</v>
-      </c>
+          <t>Light-duty servo (handout §2 table)</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
       <c r="J47" s="6" t="inlineStr">
         <is>
           <t>units</t>
@@ -2823,9 +2825,10 @@
       </c>
       <c r="K47" s="9" t="n"/>
       <c r="L47" s="10" t="n"/>
-      <c r="M47" s="11">
-        <f>IF(K47="","",MAX(0,I47-K47))</f>
-        <v/>
+      <c r="M47" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N47" s="6" t="inlineStr"/>
     </row>
@@ -2837,35 +2840,35 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Flutesan 10 kΩ trim potentiometer with knob (12 pc)</t>
+          <t>URBEST roller-lever micro switch, SPDT (10-pack)</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>B09G9TBY38</t>
+          <t>B00MFRMFS6</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>4 packs = 40</t>
         </is>
       </c>
       <c r="E48" s="6" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>7.99</v>
+        <v>27.96</v>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>Handout POT_PIN</t>
+          <t>Handout LIMIT_SWITCH_PIN; joint homing</t>
         </is>
       </c>
       <c r="H48" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -2888,28 +2891,28 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Geekworm UNO case, clear ABS</t>
+          <t>Flutesan 10 kΩ trim potentiometer with knob (12 pc)</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>B01C8500L8</t>
+          <t>B09G9TBY38</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>25</v>
+        <v>7.99</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Controller enclosure</t>
+          <t>Handout POT_PIN</t>
         </is>
       </c>
       <c r="H49" s="6" t="n">
@@ -2939,12 +2942,12 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>NexiGo N60 1080p webcam</t>
+          <t>Geekworm UNO case, clear ABS</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>B088TSR6YJ</t>
+          <t>B01C8500L8</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -2956,11 +2959,11 @@
         <v>5</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>124.95</v>
+        <v>25</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>Machine vision (Phase 3)</t>
+          <t>Controller enclosure</t>
         </is>
       </c>
       <c r="H50" s="6" t="n">
@@ -2990,28 +2993,28 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>UGREEN Revodok 105 USB-C hub, 5-in-1</t>
+          <t>NexiGo N60 1080p webcam</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>B0BR3M8XHK</t>
+          <t>B088TSR6YJ</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E51" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>79.89</v>
+        <v>124.95</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Laptop: webcam + Arduino</t>
+          <t>Machine vision (Phase 3)</t>
         </is>
       </c>
       <c r="H51" s="6" t="n">
@@ -3041,28 +3044,28 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>TAKAGI USB-A to USB-C cable, 6 ft (3-pack)</t>
+          <t>UGREEN Revodok 105 USB-C hub, 5-in-1</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>B07SMNZK8H</t>
+          <t>B0BR3M8XHK</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>4 packs = 12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E52" s="6" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>36.96</v>
+        <v>79.89</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>Uno Q programming (USB-C)</t>
+          <t>Laptop: webcam + Arduino</t>
         </is>
       </c>
       <c r="H52" s="6" t="n">
@@ -3092,32 +3095,36 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>USB-C 20 W charger block (4-pack)</t>
+          <t>TAKAGI USB-A to USB-C cable, 6 ft (3-pack)</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>B0B2WLSY9D</t>
+          <t>B07SMNZK8H</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>4 packs = 12</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>9.98</v>
+        <v>36.96</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Probably powers the Uno Q off-laptop</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
+          <t>Uno Q programming (USB-C)</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I53" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
           <t>units</t>
@@ -3125,10 +3132,9 @@
       </c>
       <c r="K53" s="9" t="n"/>
       <c r="L53" s="10" t="n"/>
-      <c r="M53" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M53" s="11">
+        <f>IF(K53="","",MAX(0,I53-K53))</f>
+        <v/>
       </c>
       <c r="N53" s="6" t="inlineStr"/>
     </row>
@@ -3140,36 +3146,32 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>ELEGOO 400-point breadboard (6-pack)</t>
+          <t>USB-C 20 W charger block (4-pack)</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>B0CYPVMK9J</t>
+          <t>B0B2WLSY9D</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>2 packs = 12</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E54" s="6" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>15.88</v>
+        <v>9.98</v>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>Phase 1 wiring</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I54" s="6" t="n">
-        <v>9</v>
-      </c>
+          <t>Probably powers the Uno Q off-laptop</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="n"/>
       <c r="J54" s="6" t="inlineStr">
         <is>
           <t>units</t>
@@ -3177,9 +3179,10 @@
       </c>
       <c r="K54" s="9" t="n"/>
       <c r="L54" s="10" t="n"/>
-      <c r="M54" s="11">
-        <f>IF(K54="","",MAX(0,I54-K54))</f>
-        <v/>
+      <c r="M54" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N54" s="6" t="inlineStr"/>
     </row>
@@ -3191,24 +3194,24 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>MCIGICM 830-point breadboard (10-pack)</t>
+          <t>ELEGOO 400-point breadboard (6-pack)</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>B07H9X7XVN</t>
+          <t>B0CYPVMK9J</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2 packs = 12</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>19.99</v>
+        <v>15.88</v>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
@@ -3242,41 +3245,46 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>EDGELEC jumper wires M–F, 20 cm (120 pc)</t>
+          <t>MCIGICM 830-point breadboard (10-pack)</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>B07GD2BWPY</t>
+          <t>B07H9X7XVN</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>2 packs</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="n"/>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="F56" s="8" t="n">
-        <v>12.86</v>
+        <v>19.99</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>Wiring</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="n"/>
-      <c r="I56" s="6" t="n"/>
+          <t>Phase 1 wiring</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>packs</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K56" s="9" t="n"/>
       <c r="L56" s="10" t="n"/>
-      <c r="M56" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M56" s="11">
+        <f>IF(K56="","",MAX(0,I56-K56))</f>
+        <v/>
       </c>
       <c r="N56" s="6" t="inlineStr"/>
     </row>
@@ -3288,22 +3296,22 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>EDGELEC jumper wires M–M, 20 cm (120 pc)</t>
+          <t>EDGELEC jumper wires M–F, 20 cm (120 pc)</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>B07GD3JVHD</t>
+          <t>B07GD2BWPY</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>1 pack</t>
+          <t>2 packs</t>
         </is>
       </c>
       <c r="E57" s="6" t="n"/>
       <c r="F57" s="8" t="n">
-        <v>7.98</v>
+        <v>12.86</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -3334,12 +3342,12 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>ELEGOO Dupont jumper kit M–F / M–M / F–F (120 pc)</t>
+          <t>EDGELEC jumper wires M–M, 20 cm (120 pc)</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>B01EV70C78</t>
+          <t>B07GD3JVHD</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
@@ -3349,7 +3357,7 @@
       </c>
       <c r="E58" s="6" t="n"/>
       <c r="F58" s="8" t="n">
-        <v>6.88</v>
+        <v>7.98</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -3380,24 +3388,22 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>TUOFENG 22 AWG solid hookup wire, 6 colors × 30 ft</t>
+          <t>ELEGOO Dupont jumper kit M–F / M–M / F–F (120 pc)</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>B07TX6BX47</t>
+          <t>B01EV70C78</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>1</v>
-      </c>
+          <t>1 pack</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n"/>
       <c r="F59" s="8" t="n">
-        <v>15.1</v>
+        <v>6.88</v>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
@@ -3408,7 +3414,7 @@
       <c r="I59" s="6" t="n"/>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>spools</t>
+          <t>packs</t>
         </is>
       </c>
       <c r="K59" s="9" t="n"/>
@@ -3428,12 +3434,12 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>4-conductor 22 AWG cable, 40 ft</t>
+          <t>TUOFENG 22 AWG solid hookup wire, 6 colors × 30 ft</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>B0793NGKL9</t>
+          <t>B07TX6BX47</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
@@ -3445,11 +3451,11 @@
         <v>1</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>14.98</v>
+        <v>15.1</v>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>Stepper lead extensions up the arm</t>
+          <t>Wiring</t>
         </is>
       </c>
       <c r="H60" s="6" t="n"/>
@@ -3476,35 +3482,35 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>DaFuRui 4-pin 5.08 mm pluggable screw terminal (15 pairs)</t>
+          <t>4-conductor 22 AWG cable, 40 ft</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>B0C2Y3VSVB</t>
+          <t>B0793NGKL9</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E61" s="6" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>16.99</v>
+        <v>14.98</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Motor connectors</t>
+          <t>Stepper lead extensions up the arm</t>
         </is>
       </c>
       <c r="H61" s="6" t="n"/>
       <c r="I61" s="6" t="n"/>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>spools</t>
         </is>
       </c>
       <c r="K61" s="9" t="n"/>
@@ -3524,35 +3530,35 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Goupchn banana plug to breadboard leads</t>
+          <t>DaFuRui 4-pin 5.08 mm pluggable screw terminal (15 pairs)</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>B08KZKGWTJ</t>
+          <t>B0C2Y3VSVB</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E62" s="6" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>17.62</v>
+        <v>16.99</v>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>Bench supply to breadboard</t>
+          <t>Motor connectors</t>
         </is>
       </c>
       <c r="H62" s="6" t="n"/>
       <c r="I62" s="6" t="n"/>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>packs</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K62" s="9" t="n"/>
@@ -3572,33 +3578,35 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>BOJACK resistor kit, 25 values (1000 pc)</t>
+          <t>Goupchn banana plug to breadboard leads</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>B08FD1XVL6</t>
+          <t>B08KZKGWTJ</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="n"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>2</v>
+      </c>
       <c r="F63" s="8" t="n">
-        <v>9.890000000000001</v>
+        <v>17.62</v>
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>LEDs, pull-ups</t>
+          <t>Bench supply to breadboard</t>
         </is>
       </c>
       <c r="H63" s="6" t="n"/>
       <c r="I63" s="6" t="n"/>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>kits</t>
+          <t>packs</t>
         </is>
       </c>
       <c r="K63" s="9" t="n"/>
@@ -3613,51 +3621,46 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>Tools (reusable)</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Bondhus 10686 ball-end hex screwdriver set, 1.5–5 mm</t>
+          <t>BOJACK resistor kit, 25 values (1000 pc)</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>B0006O4AD8</t>
+          <t>B08FD1XVL6</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>5 sets</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="n">
-        <v>5</v>
-      </c>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="n"/>
       <c r="F64" s="8" t="n">
-        <v>84.2</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>1 per team plus a spare: 9 sets needed, so buy 4 more</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I64" s="6" t="n">
-        <v>9</v>
-      </c>
+          <t>LEDs, pull-ups</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="n"/>
+      <c r="I64" s="6" t="n"/>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>sets</t>
+          <t>kits</t>
         </is>
       </c>
       <c r="K64" s="9" t="n"/>
       <c r="L64" s="10" t="n"/>
-      <c r="M64" s="11">
-        <f>IF(K64="","",MAX(0,I64-K64))</f>
-        <v/>
+      <c r="M64" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N64" s="6" t="inlineStr"/>
     </row>
@@ -3669,39 +3672,46 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>AstroAI digital multimeter</t>
+          <t>Bondhus 10686 ball-end hex screwdriver set, 1.5–5 mm</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>B01ISAMUA6</t>
+          <t>B0006O4AD8</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5 sets</t>
         </is>
       </c>
       <c r="E65" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F65" s="8" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>1 per team plus a spare: 9 sets needed, so buy 4 more</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="F65" s="8" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="G65" s="6" t="inlineStr"/>
-      <c r="H65" s="6" t="n"/>
-      <c r="I65" s="6" t="n"/>
+      <c r="I65" s="6" t="n">
+        <v>9</v>
+      </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>units</t>
+          <t>sets</t>
         </is>
       </c>
       <c r="K65" s="9" t="n"/>
       <c r="L65" s="10" t="n"/>
-      <c r="M65" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="M65" s="11">
+        <f>IF(K65="","",MAX(0,I65-K65))</f>
+        <v/>
       </c>
       <c r="N65" s="6" t="inlineStr"/>
     </row>
@@ -3713,12 +3723,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Adoric 6" digital caliper</t>
+          <t>AstroAI digital multimeter</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>B07DFFYCXS</t>
+          <t>B01ISAMUA6</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -3730,7 +3740,7 @@
         <v>1</v>
       </c>
       <c r="F66" s="8" t="n">
-        <v>6.99</v>
+        <v>13.95</v>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="6" t="n"/>
@@ -3757,12 +3767,12 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>NSZETZ precision screwdriver set, 11 pc</t>
+          <t>Adoric 6" digital caliper</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>B08ZS76VDG</t>
+          <t>B07DFFYCXS</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -3774,13 +3784,9 @@
         <v>1</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>7.59</v>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>A4988 current-limit trimmer</t>
-        </is>
-      </c>
+        <v>6.99</v>
+      </c>
+      <c r="G67" s="6" t="inlineStr"/>
       <c r="H67" s="6" t="n"/>
       <c r="I67" s="6" t="n"/>
       <c r="J67" s="6" t="inlineStr">
@@ -3805,12 +3811,12 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>WGGE WG-015 wire stripper/crimper</t>
+          <t>NSZETZ precision screwdriver set, 11 pc</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>B073YG65N2</t>
+          <t>B08ZS76VDG</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -3822,9 +3828,13 @@
         <v>1</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>8.69</v>
-      </c>
-      <c r="G68" s="6" t="inlineStr"/>
+        <v>7.59</v>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>A4988 current-limit trimmer</t>
+        </is>
+      </c>
       <c r="H68" s="6" t="n"/>
       <c r="I68" s="6" t="n"/>
       <c r="J68" s="6" t="inlineStr">
@@ -3849,12 +3859,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>MAIYUM 63/37 rosin-core solder, 0.8 mm, 50 g</t>
+          <t>WGGE WG-015 wire stripper/crimper</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>B075WB98FJ</t>
+          <t>B073YG65N2</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -3866,13 +3876,9 @@
         <v>1</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
+        <v>8.69</v>
+      </c>
+      <c r="G69" s="6" t="inlineStr"/>
       <c r="H69" s="6" t="n"/>
       <c r="I69" s="6" t="n"/>
       <c r="J69" s="6" t="inlineStr">
@@ -3897,12 +3903,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Weller brass tip cleaner</t>
+          <t>MAIYUM 63/37 rosin-core solder, 0.8 mm, 50 g</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>B08FQBS97L</t>
+          <t>B075WB98FJ</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -3914,9 +3920,13 @@
         <v>1</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>10.73</v>
-      </c>
-      <c r="G70" s="6" t="inlineStr"/>
+        <v>8.9</v>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>Consumable</t>
+        </is>
+      </c>
       <c r="H70" s="6" t="n"/>
       <c r="I70" s="6" t="n"/>
       <c r="J70" s="6" t="inlineStr">
@@ -3936,35 +3946,31 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>Spare parts (not in the current CAD)</t>
+          <t>Tools (reusable)</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>uxcell 51107 thrust bearing 35×52×12 (2-pack)</t>
+          <t>Weller brass tip cleaner</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>B07G847G75</t>
+          <t>B08FQBS97L</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>9.279999999999999</v>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>CAD uses 51108</t>
-        </is>
-      </c>
+        <v>10.73</v>
+      </c>
+      <c r="G71" s="6" t="inlineStr"/>
       <c r="H71" s="6" t="n"/>
       <c r="I71" s="6" t="n"/>
       <c r="J71" s="6" t="inlineStr">
@@ -3989,28 +3995,28 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>uxcell 6802-2RS 15×24×5 (10-pack)</t>
+          <t>uxcell 51107 thrust bearing 35×52×12 (2-pack)</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>B07FVZKBKX</t>
+          <t>B07G847G75</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>2 packs = 20</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>18.76</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>Not in CAD</t>
+          <t>CAD uses 51108</t>
         </is>
       </c>
       <c r="H72" s="6" t="n"/>
@@ -4037,28 +4043,28 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>uxcell 625-2RS 5×16×5 (5-pack)</t>
+          <t>uxcell 6802-2RS 15×24×5 (10-pack)</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>B07TNNX9YX</t>
+          <t>B07FVZKBKX</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>3 packs = 15</t>
+          <t>2 packs = 20</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>21.18</v>
+        <v>18.76</v>
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Not in CAD (5 mm bore: an idler variant?)</t>
+          <t>Not in CAD</t>
         </is>
       </c>
       <c r="H73" s="6" t="n"/>
@@ -4085,28 +4091,28 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>uxcell 686-2RS 6×13×5 (20-pack)</t>
+          <t>uxcell 625-2RS 5×16×5 (5-pack)</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>B0DCP3V3B5</t>
+          <t>B07TNNX9YX</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>3 packs = 60</t>
+          <t>3 packs = 15</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>44.73</v>
+        <v>21.18</v>
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>Not in CAD (6 mm bore: planet bearings instead of bushings?)</t>
+          <t>Not in CAD (5 mm bore: an idler variant?)</t>
         </is>
       </c>
       <c r="H74" s="6" t="n"/>
@@ -4133,28 +4139,28 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>uxcell 6×35 mm dowel pin (30-pack)</t>
+          <t>uxcell 686-2RS 6×13×5 (20-pack)</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>B0F3JPNX6R</t>
+          <t>B0DCP3V3B5</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>3 packs = 60</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>11.29</v>
+        <v>44.73</v>
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>CAD uses 6×22 and 6×30</t>
+          <t>Not in CAD (6 mm bore: planet bearings instead of bushings?)</t>
         </is>
       </c>
       <c r="H75" s="6" t="n"/>
@@ -4181,28 +4187,28 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>ruthex M4 × 8.1 heat-set insert (50-pack)</t>
+          <t>uxcell 6×35 mm dowel pin (30-pack)</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>B07YSV66Y5</t>
+          <t>B0F3JPNX6R</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>30</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>9.49</v>
+        <v>11.29</v>
       </c>
       <c r="G76" s="6" t="inlineStr">
         <is>
-          <t>CAD uses only M3 and M5 inserts</t>
+          <t>CAD uses 6×22 and 6×30</t>
         </is>
       </c>
       <c r="H76" s="6" t="n"/>
@@ -4229,33 +4235,35 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Kadrick M4 assortment, 6–40 mm (1400 pc)</t>
+          <t>ruthex M4 × 8.1 heat-set insert (50-pack)</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>B0CQNPWSG4</t>
+          <t>B07YSV66Y5</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>1 kit</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="n"/>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>50</v>
+      </c>
       <c r="F77" s="8" t="n">
-        <v>22.99</v>
+        <v>9.49</v>
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>CAD has no M4 screws (only the set screw)</t>
+          <t>CAD uses only M3 and M5 inserts</t>
         </is>
       </c>
       <c r="H77" s="6" t="n"/>
       <c r="I77" s="6" t="n"/>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>kits</t>
+          <t>units</t>
         </is>
       </c>
       <c r="K77" s="9" t="n"/>
@@ -4267,37 +4275,84 @@
       </c>
       <c r="N77" s="6" t="inlineStr"/>
     </row>
-    <row r="79">
-      <c r="E79" s="15" t="inlineStr">
-        <is>
-          <t>Total spent</t>
-        </is>
-      </c>
-      <c r="F79" s="16">
-        <f>SUM(F6:F77)</f>
-        <v/>
-      </c>
-    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>Spare parts (not in the current CAD)</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Kadrick M4 assortment, 6–40 mm (1400 pc)</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>B0CQNPWSG4</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>1 kit</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="8" t="n">
+        <v>22.99</v>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>CAD has no M4 screws (only the set screw)</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="n"/>
+      <c r="I78" s="6" t="n"/>
+      <c r="J78" s="6" t="inlineStr">
+        <is>
+          <t>kits</t>
+        </is>
+      </c>
+      <c r="K78" s="9" t="n"/>
+      <c r="L78" s="10" t="n"/>
+      <c r="M78" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79"/>
     <row r="80">
       <c r="E80" s="15" t="inlineStr">
         <is>
+          <t>Total spent</t>
+        </is>
+      </c>
+      <c r="F80" s="16">
+        <f>SUM(F6:F78)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="E81" s="15" t="inlineStr">
+        <is>
           <t>Rows counted</t>
         </is>
       </c>
-      <c r="F80" s="15">
-        <f>COUNT(K6:K77)&amp;" of "&amp;ROWS(K6:K77)</f>
+      <c r="F81" s="15">
+        <f>COUNT(K6:K78)&amp;" of "&amp;ROWS(K6:K78)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N77"/>
+  <autoFilter ref="A5:N78"/>
   <mergeCells count="3">
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K6:K77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Count" error="Enter a number (0 or more)." type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="K6:K78" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Count" error="Enter a number (0 or more)." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -4325,54 +4380,54 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId71"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Fix I-25: thicker NEMA17 mount puts the set screw on the shaft flat
The course NEMA17's shaft is round for about 10 mm before its D-flat, so
with the 10 mm mount the input-shaft set screw (z 16.8) bore on the round
part. Replace the mount with the instructor's 18 mm Fusion part
(STEP/imported/fusion/NEMA17_thicker_mount.step): motor face z 24 -> 32,
flat now z 23.3..8.3. Ø3.3 holes (FIT.m3_clear), Ø7 x 3 motor-screw
counterbores, Ø7 radial hole at z 19.5.

- planetary_gearbox takes MOTOR_FACE_Z from the mount.
- fusion_map: mount gated against the new STEP, PASS 0.003 % symdiff.
- Interference: no new pair. J1/J2 clearance unchanged.
- Screws: M3 x 22 mount -> back cover, M3 x 18 motor (inventory.md,
  inventory.xlsx N29).
- design.md part row, power path, I-25; migration log Session 10;
  re-rendered joint12_iso, robot_arm_zero, robot_arm_pick.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -612,7 +612,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -1898,7 +1897,7 @@
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
-          <t>Not on Amazon: 3DJake US, ruthex GE-M3Sx40-002 (EAN 4260528721238). Same knurl as M3 × 5.7 (Ø4.6, Ø4.0 hole). Screws: M3 × 14 (not 16)</t>
+          <t>Not on Amazon: 3DJake US, ruthex GE-M3Sx40-002 (EAN 4260528721238). Same knurl as M3 × 5.7 (Ø4.6, Ø4.0 hole). Screws: M3 × 22 through the 18 mm mount (design.md I-25)</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4320,6 @@
       </c>
       <c r="N78" s="6" t="inlineStr"/>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="E80" s="15" t="inlineStr">
         <is>

</xml_diff>